<commit_message>
chuan bi file thong ke
</commit_message>
<xml_diff>
--- a/excel/read_dethi.xlsx
+++ b/excel/read_dethi.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\VISUAL\my-project\QuanLyQuiz\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{74695871-2475-4BCD-9FA1-CF537B7E9CA4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{36D975D2-FC39-4604-95A0-6F070290CA9D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{1DDF21FF-ACF5-491C-A4EC-DBC3D782DD3D}"/>
   </bookViews>
@@ -447,8 +447,9 @@
   <sheetFormatPr defaultRowHeight="18" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="22.1796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="9.36328125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="9.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="3" width="8.7265625" style="1"/>
+    <col min="4" max="4" width="9.36328125" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.81640625" style="1" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.35">

</xml_diff>